<commit_message>
Update demo Excel files in tabtools/demo
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_crosstab.xlsx
+++ b/tabtools/demo/demo_crosstab.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="195" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="194" uniqueCount="70">
   <si>
     <t>Table 16. Treatment by Sex</t>
   </si>
@@ -228,15 +228,12 @@
   <si>
     <t>2,149 (35.4%)</t>
   </si>
-  <si>
-    <t>Percentages are row percentages within each treatment group.</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="813">
+  <fonts count="666">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -2962,607 +2959,6 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <i/>
     </font>
   </fonts>
   <fills count="15">
@@ -3638,7 +3034,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="579">
+  <borders count="474">
     <border>
       <left/>
       <right/>
@@ -6831,716 +6227,11 @@
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
-    <border/>
-    <border/>
-    <border/>
-    <border/>
-    <border/>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="579">
+  <cellXfs count="474">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -9369,411 +8060,6 @@
     </xf>
     <xf numFmtId="0" fontId="665" fillId="14" borderId="473" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="474" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="475" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="476" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="477" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="478" xfId="0"/>
-    <xf numFmtId="0" fontId="667" fillId="0" borderId="479" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="669" fillId="0" borderId="480" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="671" fillId="0" borderId="481" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="673" fillId="0" borderId="482" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="675" fillId="0" borderId="483" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="677" fillId="0" borderId="484" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="679" fillId="0" borderId="485" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="681" fillId="0" borderId="486" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="683" fillId="0" borderId="487" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="685" fillId="0" borderId="488" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="687" fillId="0" borderId="489" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="689" fillId="0" borderId="490" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="691" fillId="0" borderId="491" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="693" fillId="0" borderId="492" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="695" fillId="0" borderId="493" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="697" fillId="0" borderId="494" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="699" fillId="0" borderId="495" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="701" fillId="0" borderId="496" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="703" fillId="0" borderId="497" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="705" fillId="0" borderId="498" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="707" fillId="0" borderId="499" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="709" fillId="0" borderId="500" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="711" fillId="0" borderId="501" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="713" fillId="0" borderId="502" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="715" fillId="0" borderId="503" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="717" fillId="0" borderId="504" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="719" fillId="0" borderId="505" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="721" fillId="0" borderId="506" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="723" fillId="0" borderId="507" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="725" fillId="0" borderId="508" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="727" fillId="0" borderId="509" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="729" fillId="0" borderId="510" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="731" fillId="0" borderId="511" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="733" fillId="0" borderId="512" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="735" fillId="0" borderId="513" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="737" fillId="0" borderId="514" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="739" fillId="0" borderId="515" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="741" fillId="0" borderId="516" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="743" fillId="0" borderId="517" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="745" fillId="0" borderId="518" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="747" fillId="0" borderId="519" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="748" fillId="0" borderId="520" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="749" fillId="0" borderId="521" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="750" fillId="0" borderId="522" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="751" fillId="0" borderId="523" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="752" fillId="0" borderId="524" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="753" fillId="0" borderId="525" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="754" fillId="0" borderId="526" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="755" fillId="0" borderId="527" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="756" fillId="0" borderId="528" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="757" fillId="0" borderId="529" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="758" fillId="0" borderId="530" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="760" fillId="0" borderId="531" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="762" fillId="0" borderId="532" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="764" fillId="0" borderId="533" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="766" fillId="0" borderId="534" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="767" fillId="0" borderId="535" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="768" fillId="0" borderId="536" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="769" fillId="0" borderId="537" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="770" fillId="0" borderId="538" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="771" fillId="0" borderId="539" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="772" fillId="0" borderId="540" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="773" fillId="0" borderId="541" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="774" fillId="0" borderId="542" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="775" fillId="0" borderId="543" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="776" fillId="0" borderId="544" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="777" fillId="0" borderId="545" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="778" fillId="0" borderId="546" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="779" fillId="0" borderId="547" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="780" fillId="0" borderId="548" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="781" fillId="0" borderId="549" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="782" fillId="0" borderId="550" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="783" fillId="0" borderId="551" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="784" fillId="0" borderId="552" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="785" fillId="0" borderId="553" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="786" fillId="0" borderId="554" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="787" fillId="0" borderId="555" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="788" fillId="0" borderId="556" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="789" fillId="0" borderId="557" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="790" fillId="0" borderId="558" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="791" fillId="0" borderId="559" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="792" fillId="0" borderId="560" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="793" fillId="0" borderId="561" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="794" fillId="0" borderId="562" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="795" fillId="0" borderId="563" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="796" fillId="0" borderId="564" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="797" fillId="0" borderId="565" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="798" fillId="0" borderId="566" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="799" fillId="0" borderId="567" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="800" fillId="0" borderId="568" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="801" fillId="0" borderId="569" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="802" fillId="0" borderId="570" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="803" fillId="0" borderId="571" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="804" fillId="0" borderId="572" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="805" fillId="0" borderId="573" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="806" fillId="0" borderId="574" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="807" fillId="0" borderId="575" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="808" fillId="0" borderId="576" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="810" fillId="0" borderId="577" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="812" fillId="0" borderId="578" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -10421,149 +8707,128 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="1.7109375" style="474" customWidth="true"/>
-    <col min="2" max="2" width="15.7109375" style="475" customWidth="true"/>
-    <col min="3" max="3" width="14.7109375" style="476" customWidth="true"/>
-    <col min="4" max="4" width="14.7109375" style="477" customWidth="true"/>
-    <col min="5" max="5" width="14.7109375" style="478" customWidth="true"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="522" t="s">
+      <c r="A1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="514" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="514" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="514" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="514" t="s">
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="484" t="s">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="535" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="536" t="s">
+      <c r="C2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="537" t="s">
+      <c r="D2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="538" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="489" t="s">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="490" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="539" t="s">
+      <c r="C3" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="540" t="s">
+      <c r="D3" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="541" t="s">
+      <c r="E3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="494" t="s">
+      <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="495" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="542" t="s">
+      <c r="C4" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="543" t="s">
+      <c r="D4" t="s">
         <v>69</v>
       </c>
-      <c r="E4" s="544" t="s">
+      <c r="E4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="499" t="s">
+      <c r="A5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="558" t="s">
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="559" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="560" t="s">
+      <c r="D5" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="561" t="s">
+      <c r="E5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="504" t="s">
+      <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="567" t="s">
+      <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="562" t="s">
+      <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="562" t="s">
+      <c r="D6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="562" t="s">
+      <c r="E6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="509" t="s">
+      <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="570" t="s">
+      <c r="B7" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="571" t="s">
+      <c r="C7" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="572" t="s">
+      <c r="D7" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="573" t="s">
+      <c r="E7" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="578" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="475"/>
-      <c r="D8" s="475"/>
-      <c r="E8" s="475"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B8:E8"/>
-  </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
tabtools: add demos, doc contracts test, update help files
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_crosstab.xlsx
+++ b/tabtools/demo/demo_crosstab.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="194" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="195" uniqueCount="71">
   <si>
     <t>Table 16. Treatment by Sex</t>
   </si>
@@ -228,12 +228,15 @@
   <si>
     <t>2,149 (35.4%)</t>
   </si>
+  <si>
+    <t>Percentages are row percentages within each treatment group.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="666">
+  <fonts count="813">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -2959,6 +2962,607 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <i/>
     </font>
   </fonts>
   <fills count="15">
@@ -3034,7 +3638,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="474">
+  <borders count="579">
     <border>
       <left/>
       <right/>
@@ -6227,11 +6831,716 @@
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="474">
+  <cellXfs count="579">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -8060,6 +9369,411 @@
     </xf>
     <xf numFmtId="0" fontId="665" fillId="14" borderId="473" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="474" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="475" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="476" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="477" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="478" xfId="0"/>
+    <xf numFmtId="0" fontId="667" fillId="0" borderId="479" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="669" fillId="0" borderId="480" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="671" fillId="0" borderId="481" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="673" fillId="0" borderId="482" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="675" fillId="0" borderId="483" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="677" fillId="0" borderId="484" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="679" fillId="0" borderId="485" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="681" fillId="0" borderId="486" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="683" fillId="0" borderId="487" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="685" fillId="0" borderId="488" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="687" fillId="0" borderId="489" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="689" fillId="0" borderId="490" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="691" fillId="0" borderId="491" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="693" fillId="0" borderId="492" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="695" fillId="0" borderId="493" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="697" fillId="0" borderId="494" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="699" fillId="0" borderId="495" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="701" fillId="0" borderId="496" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="703" fillId="0" borderId="497" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="705" fillId="0" borderId="498" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="707" fillId="0" borderId="499" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="709" fillId="0" borderId="500" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="711" fillId="0" borderId="501" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="713" fillId="0" borderId="502" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="715" fillId="0" borderId="503" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="717" fillId="0" borderId="504" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="719" fillId="0" borderId="505" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="721" fillId="0" borderId="506" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="723" fillId="0" borderId="507" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="725" fillId="0" borderId="508" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="727" fillId="0" borderId="509" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="729" fillId="0" borderId="510" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="731" fillId="0" borderId="511" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="733" fillId="0" borderId="512" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="735" fillId="0" borderId="513" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="737" fillId="0" borderId="514" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="739" fillId="0" borderId="515" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="741" fillId="0" borderId="516" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="743" fillId="0" borderId="517" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="745" fillId="0" borderId="518" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="747" fillId="0" borderId="519" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="748" fillId="0" borderId="520" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="749" fillId="0" borderId="521" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="750" fillId="0" borderId="522" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="751" fillId="0" borderId="523" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="752" fillId="0" borderId="524" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="753" fillId="0" borderId="525" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="754" fillId="0" borderId="526" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="755" fillId="0" borderId="527" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="756" fillId="0" borderId="528" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="757" fillId="0" borderId="529" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="758" fillId="0" borderId="530" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="760" fillId="0" borderId="531" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="762" fillId="0" borderId="532" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="764" fillId="0" borderId="533" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="766" fillId="0" borderId="534" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="767" fillId="0" borderId="535" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="768" fillId="0" borderId="536" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="769" fillId="0" borderId="537" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="770" fillId="0" borderId="538" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="771" fillId="0" borderId="539" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="772" fillId="0" borderId="540" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="773" fillId="0" borderId="541" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="774" fillId="0" borderId="542" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="775" fillId="0" borderId="543" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="776" fillId="0" borderId="544" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="777" fillId="0" borderId="545" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="778" fillId="0" borderId="546" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="779" fillId="0" borderId="547" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="780" fillId="0" borderId="548" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="781" fillId="0" borderId="549" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="782" fillId="0" borderId="550" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="783" fillId="0" borderId="551" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="784" fillId="0" borderId="552" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="785" fillId="0" borderId="553" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="786" fillId="0" borderId="554" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="787" fillId="0" borderId="555" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="788" fillId="0" borderId="556" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="789" fillId="0" borderId="557" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="790" fillId="0" borderId="558" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="791" fillId="0" borderId="559" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="792" fillId="0" borderId="560" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="793" fillId="0" borderId="561" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="794" fillId="0" borderId="562" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="795" fillId="0" borderId="563" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="796" fillId="0" borderId="564" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="797" fillId="0" borderId="565" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="798" fillId="0" borderId="566" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="799" fillId="0" borderId="567" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="800" fillId="0" borderId="568" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="801" fillId="0" borderId="569" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="802" fillId="0" borderId="570" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="803" fillId="0" borderId="571" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="804" fillId="0" borderId="572" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="805" fillId="0" borderId="573" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="806" fillId="0" borderId="574" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="807" fillId="0" borderId="575" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="808" fillId="0" borderId="576" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="810" fillId="0" borderId="577" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="812" fillId="0" borderId="578" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -8707,128 +10421,149 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="1.7109375" style="474" customWidth="true"/>
+    <col min="2" max="2" width="15.7109375" style="475" customWidth="true"/>
+    <col min="3" max="3" width="14.7109375" style="476" customWidth="true"/>
+    <col min="4" max="4" width="14.7109375" style="477" customWidth="true"/>
+    <col min="5" max="5" width="14.7109375" style="478" customWidth="true"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="522" t="s">
         <v>64</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="514" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="514" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="514" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="514" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="484" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="535" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="536" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="537" t="s">
         <v>27</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="538" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="489" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="490" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="539" t="s">
         <v>66</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="540" t="s">
         <v>68</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="541" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4" s="494" t="s">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="495" t="s">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="542" t="s">
         <v>67</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="543" t="s">
         <v>69</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="544" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" s="499" t="s">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="558" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="559" t="s">
         <v>26</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="560" t="s">
         <v>30</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="561" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
+      <c r="A6" s="504" t="s">
         <v>1</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="567" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="562" t="s">
         <v>1</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="562" t="s">
         <v>1</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="562" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s">
+      <c r="A7" s="509" t="s">
         <v>1</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="570" t="s">
         <v>65</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="571" t="s">
         <v>1</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="572" t="s">
         <v>1</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="573" t="s">
         <v>1</v>
       </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="578" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="475"/>
+      <c r="D8" s="475"/>
+      <c r="E8" s="475"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B8:E8"/>
+  </mergeCells>
 </worksheet>
 </file>
</xml_diff>